<commit_message>
feat: multi-month filter, cashflow, corrected unit costs, consolidated sales data
- app/db.py: added get_available_months, get_monthly_breakdown, get_kpis_by_months
- app/components/sidebar.py: global month filter (multiselect) wired to session_state
- app/components/monthly_block.py: reads global filter, fixed import error
- app/app.py: month-aware KPI cards
- data/parquet/products.parquet: unit_cost corrected from CSV medians (31 SKUs), ABC recomputed
- data/parquet/daily_sales.parquet: rebuilt from consolidated file (3829 units, R118845)
- data/parquet/cashflow.parquet: sales entradas + CMV + custos fixos Mar/Apr (32 rows)
- data/excel/FuloFilo_Master.xlsx: Catalog unit_cost updated, Cashflow sheet populated
- data/excel/source_sync_status.json: healthy_production_data=true
- data/suppliers/: 13 suppliers dashboard HTML + XLSX
- data/raw/custos_fixos/: fixed costs JSON R12950/month
- data/raw/: consolidated sales CSVs Mar-Apr 2026
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailySales" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cashflow" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CategoryOverrides" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DailySales" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cashflow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CategoryOverrides" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Meta" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E2" t="n">
         <v>5</v>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E4" t="n">
         <v>5</v>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
         <v>5</v>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E9" t="n">
         <v>5</v>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E10" t="n">
         <v>5</v>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E11" t="n">
         <v>5</v>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E12" t="n">
         <v>5</v>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E13" t="n">
         <v>5</v>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E14" t="n">
         <v>5</v>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E15" t="n">
         <v>5</v>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E16" t="n">
         <v>5</v>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E17" t="n">
         <v>5</v>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E18" t="n">
         <v>5</v>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E19" t="n">
         <v>5</v>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E20" t="n">
         <v>5</v>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E21" t="n">
         <v>5</v>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E22" t="n">
         <v>5</v>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E23" t="n">
         <v>5</v>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E24" t="n">
         <v>5</v>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E25" t="n">
         <v>5</v>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E26" t="n">
         <v>5</v>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E27" t="n">
         <v>5</v>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E28" t="n">
         <v>5</v>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E29" t="n">
         <v>5</v>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E30" t="n">
         <v>5</v>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2653,7 +2653,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E31" t="n">
         <v>5</v>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E32" t="n">
         <v>5</v>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E33" t="n">
         <v>5</v>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E34" t="n">
         <v>5</v>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E35" t="n">
         <v>5</v>
@@ -2802,7 +2802,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E36" t="n">
         <v>5</v>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E37" t="n">
         <v>5</v>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E38" t="n">
         <v>5</v>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E39" t="n">
         <v>5</v>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E40" t="n">
         <v>5</v>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Seeded from Mar-Apr 2026 sales history; current stock not yet confirmed.</t>
+          <t>Estoque inicial — 110 unidades por produto.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: ingest sales 2026-05-01
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H179"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -12023,6 +12023,510 @@
       <c r="H179" t="inlineStr">
         <is>
           <t>item-sales-summary-2026-04-30-2026-04-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>00423</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Canga Elastano — Flamingo</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>2</v>
+      </c>
+      <c r="E180" t="n">
+        <v>55</v>
+      </c>
+      <c r="F180" t="n">
+        <v>110</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>00409</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Canga Elastano — Tye Dye</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>3</v>
+      </c>
+      <c r="E181" t="n">
+        <v>55</v>
+      </c>
+      <c r="F181" t="n">
+        <v>165</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>00429</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Canga Algodão — Cordel</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>3</v>
+      </c>
+      <c r="E182" t="n">
+        <v>40</v>
+      </c>
+      <c r="F182" t="n">
+        <v>120</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>00430</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Canga Algodão — Eu Amo Nordeste</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>2</v>
+      </c>
+      <c r="E183" t="n">
+        <v>40</v>
+      </c>
+      <c r="F183" t="n">
+        <v>80</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+      <c r="E184" t="n">
+        <v>125</v>
+      </c>
+      <c r="F184" t="n">
+        <v>125</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>10027</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Porta lingerie</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>3</v>
+      </c>
+      <c r="E185" t="n">
+        <v>25</v>
+      </c>
+      <c r="F185" t="n">
+        <v>75</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Carteira alça</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>4</v>
+      </c>
+      <c r="E186" t="n">
+        <v>15</v>
+      </c>
+      <c r="F186" t="n">
+        <v>60</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Placa kit 100</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>2</v>
+      </c>
+      <c r="E187" t="n">
+        <v>100</v>
+      </c>
+      <c r="F187" t="n">
+        <v>200</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>5</v>
+      </c>
+      <c r="E188" t="n">
+        <v>20</v>
+      </c>
+      <c r="F188" t="n">
+        <v>100</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>10031</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Boné</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>1</v>
+      </c>
+      <c r="E189" t="n">
+        <v>60</v>
+      </c>
+      <c r="F189" t="n">
+        <v>60</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Bata infantil</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>2</v>
+      </c>
+      <c r="E190" t="n">
+        <v>44</v>
+      </c>
+      <c r="F190" t="n">
+        <v>88</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>10010</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Oxe adulto</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>2</v>
+      </c>
+      <c r="E191" t="n">
+        <v>60</v>
+      </c>
+      <c r="F191" t="n">
+        <v>120</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>10017</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Sereia</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" t="n">
+        <v>180</v>
+      </c>
+      <c r="F192" t="n">
+        <v>180</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>10018</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Vestido algodão</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>2</v>
+      </c>
+      <c r="E193" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="F193" t="n">
+        <v>119.2</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-01-2026-05-01</t>
         </is>
       </c>
     </row>
@@ -12039,7 +12543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -13059,6 +13563,36 @@
         <v>1454.85</v>
       </c>
       <c r="F34" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Vendas 2026-05-01 → 2026-05-01</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1602.2</v>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
auto: ingest sales 2026-05-02
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H207"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -12527,6 +12527,510 @@
       <c r="H193" t="inlineStr">
         <is>
           <t>item-sales-summary-2026-05-01-2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>00400</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Canga Elastano — San Andrés</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>3</v>
+      </c>
+      <c r="E194" t="n">
+        <v>55</v>
+      </c>
+      <c r="F194" t="n">
+        <v>165</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>00404</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Canga Elastano — Borboleta</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>2</v>
+      </c>
+      <c r="E195" t="n">
+        <v>55</v>
+      </c>
+      <c r="F195" t="n">
+        <v>110</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>00431</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Canga Algodão — Oxente</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>4</v>
+      </c>
+      <c r="E196" t="n">
+        <v>40</v>
+      </c>
+      <c r="F196" t="n">
+        <v>160</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>00428</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Canga Algodão — Instrumentos Musicais</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>2</v>
+      </c>
+      <c r="E197" t="n">
+        <v>40</v>
+      </c>
+      <c r="F197" t="n">
+        <v>80</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>10021</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Bolsinha 15</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>3</v>
+      </c>
+      <c r="E198" t="n">
+        <v>15</v>
+      </c>
+      <c r="F198" t="n">
+        <v>45</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>10022</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Bolsinha 20</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>2</v>
+      </c>
+      <c r="E199" t="n">
+        <v>20</v>
+      </c>
+      <c r="F199" t="n">
+        <v>40</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>10029</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 30</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>3</v>
+      </c>
+      <c r="E200" t="n">
+        <v>30</v>
+      </c>
+      <c r="F200" t="n">
+        <v>90</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>10033</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Chaveiro 5</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>5</v>
+      </c>
+      <c r="E201" t="n">
+        <v>5</v>
+      </c>
+      <c r="F201" t="n">
+        <v>25</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>10032</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Boneca</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>1</v>
+      </c>
+      <c r="E202" t="n">
+        <v>30</v>
+      </c>
+      <c r="F202" t="n">
+        <v>30</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Color 60</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>2</v>
+      </c>
+      <c r="E203" t="n">
+        <v>60</v>
+      </c>
+      <c r="F203" t="n">
+        <v>120</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>10015</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Regional infantil</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>3</v>
+      </c>
+      <c r="E204" t="n">
+        <v>45</v>
+      </c>
+      <c r="F204" t="n">
+        <v>135</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>10011</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Oxe infantil</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>2</v>
+      </c>
+      <c r="E205" t="n">
+        <v>55</v>
+      </c>
+      <c r="F205" t="n">
+        <v>110</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>10009</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Macaquinho</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" t="n">
+        <v>48</v>
+      </c>
+      <c r="F206" t="n">
+        <v>48</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>10016</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Saída praia</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>2</v>
+      </c>
+      <c r="E207" t="n">
+        <v>65</v>
+      </c>
+      <c r="F207" t="n">
+        <v>130</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-05-02-2026-05-02</t>
         </is>
       </c>
     </row>
@@ -12543,7 +13047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -13593,6 +14097,36 @@
         <v>1602.2</v>
       </c>
       <c r="F35" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Vendas 2026-05-02 → 2026-05-02</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1288</v>
+      </c>
+      <c r="F36" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
auto: ingest sales 2026-04-23
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -8666,21 +8666,546 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="15" customHeight="1" s="1"/>
-    <row r="102" ht="15" customHeight="1" s="1"/>
-    <row r="103" ht="15" customHeight="1" s="1"/>
-    <row r="104" ht="15" customHeight="1" s="1"/>
-    <row r="105" ht="15" customHeight="1" s="1"/>
-    <row r="106" ht="15" customHeight="1" s="1"/>
-    <row r="107" ht="15" customHeight="1" s="1"/>
-    <row r="108" ht="15" customHeight="1" s="1"/>
-    <row r="109" ht="15" customHeight="1" s="1"/>
-    <row r="110" ht="15" customHeight="1" s="1"/>
-    <row r="111" ht="15" customHeight="1" s="1"/>
-    <row r="112" ht="15" customHeight="1" s="1"/>
-    <row r="113" ht="15" customHeight="1" s="1"/>
-    <row r="114" ht="15" customHeight="1" s="1"/>
-    <row r="115" ht="15" customHeight="1" s="1"/>
+    <row r="101" ht="15" customHeight="1" s="1">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Bata adulto</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" t="n">
+        <v>60</v>
+      </c>
+      <c r="F101" t="n">
+        <v>60</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1" s="1">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" t="n">
+        <v>35</v>
+      </c>
+      <c r="F102" t="n">
+        <v>35</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15" customHeight="1" s="1">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" t="n">
+        <v>125</v>
+      </c>
+      <c r="F103" t="n">
+        <v>125</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15" customHeight="1" s="1">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Caneca louça</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>6</v>
+      </c>
+      <c r="E104" t="n">
+        <v>35</v>
+      </c>
+      <c r="F104" t="n">
+        <v>210</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1" s="1">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>4</v>
+      </c>
+      <c r="E105" t="n">
+        <v>20</v>
+      </c>
+      <c r="F105" t="n">
+        <v>80</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15" customHeight="1" s="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10029</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 30</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" t="n">
+        <v>30</v>
+      </c>
+      <c r="F106" t="n">
+        <v>30</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1" s="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" t="n">
+        <v>55</v>
+      </c>
+      <c r="F107" t="n">
+        <v>55</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1" s="1">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10033</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Chaveiro 5</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" t="n">
+        <v>5</v>
+      </c>
+      <c r="F108" t="n">
+        <v>5</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="1">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>39</v>
+      </c>
+      <c r="E109" t="n">
+        <v>10</v>
+      </c>
+      <c r="F109" t="n">
+        <v>390</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1" s="1">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10008</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Color XG 65</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" t="n">
+        <v>65</v>
+      </c>
+      <c r="F110" t="n">
+        <v>65</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="15" customHeight="1" s="1">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Ecobag</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>2</v>
+      </c>
+      <c r="E111" t="n">
+        <v>25</v>
+      </c>
+      <c r="F111" t="n">
+        <v>50</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="15" customHeight="1" s="1">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10035</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Imã 15</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>7</v>
+      </c>
+      <c r="E112" t="n">
+        <v>15</v>
+      </c>
+      <c r="F112" t="n">
+        <v>105</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="15" customHeight="1" s="1">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>10</v>
+      </c>
+      <c r="E113" t="n">
+        <v>20</v>
+      </c>
+      <c r="F113" t="n">
+        <v>200</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="15" customHeight="1" s="1">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>9</v>
+      </c>
+      <c r="E114" t="n">
+        <v>20</v>
+      </c>
+      <c r="F114" t="n">
+        <v>180</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="15" customHeight="1" s="1">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>13</v>
+      </c>
+      <c r="E115" t="n">
+        <v>55</v>
+      </c>
+      <c r="F115" t="n">
+        <v>715</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-23-2026-04-23</t>
+        </is>
+      </c>
+    </row>
     <row r="116" ht="15" customHeight="1" s="1"/>
     <row r="117" ht="15" customHeight="1" s="1"/>
     <row r="118" ht="15" customHeight="1" s="1"/>
@@ -8703,7 +9228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -9813,6 +10338,36 @@
         <v>3210</v>
       </c>
       <c r="F37" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Vendas 2026-04-23 → 2026-04-23</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2305</v>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
auto: ingest sales 2026-04-24
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H115"/>
+  <dimension ref="A1:H132"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -9206,15 +9206,618 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="15" customHeight="1" s="1"/>
-    <row r="117" ht="15" customHeight="1" s="1"/>
-    <row r="118" ht="15" customHeight="1" s="1"/>
-    <row r="119" ht="15" customHeight="1" s="1"/>
-    <row r="120" ht="15" customHeight="1" s="1"/>
-    <row r="121" ht="15" customHeight="1" s="1"/>
-    <row r="122" ht="15" customHeight="1" s="1"/>
-    <row r="123" ht="15" customHeight="1" s="1"/>
-    <row r="124" ht="15" customHeight="1" s="1"/>
+    <row r="116" ht="15" customHeight="1" s="1">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Bata adulto</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" t="n">
+        <v>60</v>
+      </c>
+      <c r="F116" t="n">
+        <v>60</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="15" customHeight="1" s="1">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>2</v>
+      </c>
+      <c r="E117" t="n">
+        <v>35</v>
+      </c>
+      <c r="F117" t="n">
+        <v>70</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="15" customHeight="1" s="1">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" t="n">
+        <v>125</v>
+      </c>
+      <c r="F118" t="n">
+        <v>125</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="15" customHeight="1" s="1">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10021</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Bolsinha 15</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>1</v>
+      </c>
+      <c r="E119" t="n">
+        <v>15</v>
+      </c>
+      <c r="F119" t="n">
+        <v>15</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="15" customHeight="1" s="1">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Caneca louça</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>2</v>
+      </c>
+      <c r="E120" t="n">
+        <v>35</v>
+      </c>
+      <c r="F120" t="n">
+        <v>70</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="15" customHeight="1" s="1">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>3</v>
+      </c>
+      <c r="E121" t="n">
+        <v>20</v>
+      </c>
+      <c r="F121" t="n">
+        <v>60</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="15" customHeight="1" s="1">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>3</v>
+      </c>
+      <c r="E122" t="n">
+        <v>55</v>
+      </c>
+      <c r="F122" t="n">
+        <v>165</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="15" customHeight="1" s="1">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Carteira alça</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>8</v>
+      </c>
+      <c r="E123" t="n">
+        <v>15</v>
+      </c>
+      <c r="F123" t="n">
+        <v>120</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="15" customHeight="1" s="1">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>12</v>
+      </c>
+      <c r="E124" t="n">
+        <v>10</v>
+      </c>
+      <c r="F124" t="n">
+        <v>120</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Color 60</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>2</v>
+      </c>
+      <c r="E125" t="n">
+        <v>60</v>
+      </c>
+      <c r="F125" t="n">
+        <v>120</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>10035</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Imã 15</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>5</v>
+      </c>
+      <c r="E126" t="n">
+        <v>15</v>
+      </c>
+      <c r="F126" t="n">
+        <v>75</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>17</v>
+      </c>
+      <c r="E127" t="n">
+        <v>20</v>
+      </c>
+      <c r="F127" t="n">
+        <v>340</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>11</v>
+      </c>
+      <c r="E128" t="n">
+        <v>20</v>
+      </c>
+      <c r="F128" t="n">
+        <v>220</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Placa kit 100</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>1</v>
+      </c>
+      <c r="E129" t="n">
+        <v>100</v>
+      </c>
+      <c r="F129" t="n">
+        <v>100</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>10027</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Porta lingerie</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>1</v>
+      </c>
+      <c r="E130" t="n">
+        <v>25</v>
+      </c>
+      <c r="F130" t="n">
+        <v>25</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>11</v>
+      </c>
+      <c r="E131" t="n">
+        <v>55</v>
+      </c>
+      <c r="F131" t="n">
+        <v>605</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>10018</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Vestido algodão</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>2</v>
+      </c>
+      <c r="E132" t="n">
+        <v>60</v>
+      </c>
+      <c r="F132" t="n">
+        <v>120</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9228,7 +9831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -10368,6 +10971,36 @@
         <v>2305</v>
       </c>
       <c r="F38" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Vendas 2026-04-24 → 2026-04-24</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
auto: ingest sales 2026-04-25
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H132"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -9815,6 +9815,798 @@
       <c r="H132" t="inlineStr">
         <is>
           <t>item-sales-summary-2026-04-24-2026-04-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Bata adulto</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+      <c r="E133" t="n">
+        <v>60</v>
+      </c>
+      <c r="F133" t="n">
+        <v>60</v>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Bata infantil</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" t="n">
+        <v>45</v>
+      </c>
+      <c r="F134" t="n">
+        <v>45</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>10002</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Bata XG 65</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>1</v>
+      </c>
+      <c r="E135" t="n">
+        <v>65</v>
+      </c>
+      <c r="F135" t="n">
+        <v>65</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>2</v>
+      </c>
+      <c r="E136" t="n">
+        <v>35</v>
+      </c>
+      <c r="F136" t="n">
+        <v>70</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>10020</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Bolsa 55</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>1</v>
+      </c>
+      <c r="E137" t="n">
+        <v>55</v>
+      </c>
+      <c r="F137" t="n">
+        <v>55</v>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>4</v>
+      </c>
+      <c r="E138" t="n">
+        <v>125</v>
+      </c>
+      <c r="F138" t="n">
+        <v>500</v>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Caneca louça</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>6</v>
+      </c>
+      <c r="E139" t="n">
+        <v>35</v>
+      </c>
+      <c r="F139" t="n">
+        <v>210</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>4</v>
+      </c>
+      <c r="E140" t="n">
+        <v>20</v>
+      </c>
+      <c r="F140" t="n">
+        <v>80</v>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>1</v>
+      </c>
+      <c r="E141" t="n">
+        <v>55</v>
+      </c>
+      <c r="F141" t="n">
+        <v>55</v>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Carteira alça</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>4</v>
+      </c>
+      <c r="E142" t="n">
+        <v>15</v>
+      </c>
+      <c r="F142" t="n">
+        <v>60</v>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>45</v>
+      </c>
+      <c r="E143" t="n">
+        <v>10</v>
+      </c>
+      <c r="F143" t="n">
+        <v>450</v>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Color 60</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>1</v>
+      </c>
+      <c r="E144" t="n">
+        <v>60</v>
+      </c>
+      <c r="F144" t="n">
+        <v>60</v>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>10008</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Color XG 65</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+      <c r="E145" t="n">
+        <v>65</v>
+      </c>
+      <c r="F145" t="n">
+        <v>65</v>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Ecobag</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>4</v>
+      </c>
+      <c r="E146" t="n">
+        <v>25</v>
+      </c>
+      <c r="F146" t="n">
+        <v>100</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Embalagem presente 5</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>5</v>
+      </c>
+      <c r="E147" t="n">
+        <v>5</v>
+      </c>
+      <c r="F147" t="n">
+        <v>25</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>10035</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Imã 15</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" t="n">
+        <v>15</v>
+      </c>
+      <c r="F148" t="n">
+        <v>15</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>8</v>
+      </c>
+      <c r="E149" t="n">
+        <v>20</v>
+      </c>
+      <c r="F149" t="n">
+        <v>160</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>8</v>
+      </c>
+      <c r="E150" t="n">
+        <v>20</v>
+      </c>
+      <c r="F150" t="n">
+        <v>160</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Placa kit 100</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" t="n">
+        <v>100</v>
+      </c>
+      <c r="F151" t="n">
+        <v>100</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10027</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Porta lingerie</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+      <c r="E152" t="n">
+        <v>25</v>
+      </c>
+      <c r="F152" t="n">
+        <v>25</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>12</v>
+      </c>
+      <c r="E153" t="n">
+        <v>55</v>
+      </c>
+      <c r="F153" t="n">
+        <v>660</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>10018</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Vestido algodão</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+      <c r="E154" t="n">
+        <v>60</v>
+      </c>
+      <c r="F154" t="n">
+        <v>60</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-25-2026-04-25</t>
         </is>
       </c>
     </row>
@@ -9831,7 +10623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -11001,6 +11793,36 @@
         <v>2410</v>
       </c>
       <c r="F39" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Vendas 2026-04-25 → 2026-04-25</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3080</v>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
auto: ingest sales 2026-04-26
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H154"/>
+  <dimension ref="A1:H179"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -10607,6 +10607,906 @@
       <c r="H154" t="inlineStr">
         <is>
           <t>item-sales-summary-2026-04-25-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Bata infantil</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+      <c r="E155" t="n">
+        <v>45</v>
+      </c>
+      <c r="F155" t="n">
+        <v>45</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>3</v>
+      </c>
+      <c r="E156" t="n">
+        <v>35</v>
+      </c>
+      <c r="F156" t="n">
+        <v>105</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>10004</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Body conjunto</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" t="n">
+        <v>60</v>
+      </c>
+      <c r="F157" t="n">
+        <v>60</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>10020</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Bolsa 55</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>2</v>
+      </c>
+      <c r="E158" t="n">
+        <v>55</v>
+      </c>
+      <c r="F158" t="n">
+        <v>110</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+      <c r="E159" t="n">
+        <v>125</v>
+      </c>
+      <c r="F159" t="n">
+        <v>125</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Caneca louça</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" t="n">
+        <v>35</v>
+      </c>
+      <c r="F160" t="n">
+        <v>35</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>1</v>
+      </c>
+      <c r="E161" t="n">
+        <v>20</v>
+      </c>
+      <c r="F161" t="n">
+        <v>20</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>10029</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 30</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" t="n">
+        <v>30</v>
+      </c>
+      <c r="F162" t="n">
+        <v>30</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>5</v>
+      </c>
+      <c r="E163" t="n">
+        <v>55</v>
+      </c>
+      <c r="F163" t="n">
+        <v>275</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Carteira alça</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>8</v>
+      </c>
+      <c r="E164" t="n">
+        <v>15</v>
+      </c>
+      <c r="F164" t="n">
+        <v>120</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>35</v>
+      </c>
+      <c r="E165" t="n">
+        <v>10</v>
+      </c>
+      <c r="F165" t="n">
+        <v>350</v>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Color 60</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>3</v>
+      </c>
+      <c r="E166" t="n">
+        <v>60</v>
+      </c>
+      <c r="F166" t="n">
+        <v>180</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>10008</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Color XG 65</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>1</v>
+      </c>
+      <c r="E167" t="n">
+        <v>65</v>
+      </c>
+      <c r="F167" t="n">
+        <v>65</v>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Ecobag</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E168" t="n">
+        <v>25</v>
+      </c>
+      <c r="F168" t="n">
+        <v>25</v>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Embalagem presente 5</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>2</v>
+      </c>
+      <c r="E169" t="n">
+        <v>5</v>
+      </c>
+      <c r="F169" t="n">
+        <v>10</v>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>10035</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Imã 15</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>6</v>
+      </c>
+      <c r="E170" t="n">
+        <v>15</v>
+      </c>
+      <c r="F170" t="n">
+        <v>90</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>10009</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Macaquinho</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>3</v>
+      </c>
+      <c r="E171" t="n">
+        <v>50</v>
+      </c>
+      <c r="F171" t="n">
+        <v>150</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>14</v>
+      </c>
+      <c r="E172" t="n">
+        <v>20</v>
+      </c>
+      <c r="F172" t="n">
+        <v>280</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>10012</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Oxe conjunto</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>1</v>
+      </c>
+      <c r="E173" t="n">
+        <v>80</v>
+      </c>
+      <c r="F173" t="n">
+        <v>80</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>22</v>
+      </c>
+      <c r="E174" t="n">
+        <v>20</v>
+      </c>
+      <c r="F174" t="n">
+        <v>440</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Placa kit 100</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>3</v>
+      </c>
+      <c r="E175" t="n">
+        <v>100</v>
+      </c>
+      <c r="F175" t="n">
+        <v>300</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>10027</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Porta lingerie</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>1</v>
+      </c>
+      <c r="E176" t="n">
+        <v>25</v>
+      </c>
+      <c r="F176" t="n">
+        <v>25</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>13</v>
+      </c>
+      <c r="E177" t="n">
+        <v>55</v>
+      </c>
+      <c r="F177" t="n">
+        <v>715</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>10015</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Regional infantil</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>1</v>
+      </c>
+      <c r="E178" t="n">
+        <v>45</v>
+      </c>
+      <c r="F178" t="n">
+        <v>45</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>10017</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Sereia</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>1</v>
+      </c>
+      <c r="E179" t="n">
+        <v>180</v>
+      </c>
+      <c r="F179" t="n">
+        <v>180</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-26-2026-04-26</t>
         </is>
       </c>
     </row>
@@ -10623,7 +11523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -11823,6 +12723,36 @@
         <v>3080</v>
       </c>
       <c r="F40" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Vendas 2026-04-26 → 2026-04-26</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>3860</v>
+      </c>
+      <c r="F41" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
auto: ingest sales 2026-04-27
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -4835,7 +4835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H179"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -11507,6 +11507,510 @@
       <c r="H179" t="inlineStr">
         <is>
           <t>item-sales-summary-2026-04-26-2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>2</v>
+      </c>
+      <c r="E180" t="n">
+        <v>35</v>
+      </c>
+      <c r="F180" t="n">
+        <v>70</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>2</v>
+      </c>
+      <c r="E181" t="n">
+        <v>125</v>
+      </c>
+      <c r="F181" t="n">
+        <v>250</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>3</v>
+      </c>
+      <c r="E182" t="n">
+        <v>20</v>
+      </c>
+      <c r="F182" t="n">
+        <v>60</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>1</v>
+      </c>
+      <c r="E183" t="n">
+        <v>55</v>
+      </c>
+      <c r="F183" t="n">
+        <v>55</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>4</v>
+      </c>
+      <c r="E184" t="n">
+        <v>10</v>
+      </c>
+      <c r="F184" t="n">
+        <v>40</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Color 60</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>1</v>
+      </c>
+      <c r="E185" t="n">
+        <v>60</v>
+      </c>
+      <c r="F185" t="n">
+        <v>60</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Ecobag</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>3</v>
+      </c>
+      <c r="E186" t="n">
+        <v>25</v>
+      </c>
+      <c r="F186" t="n">
+        <v>75</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Embalagem presente 5</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>1</v>
+      </c>
+      <c r="E187" t="n">
+        <v>5</v>
+      </c>
+      <c r="F187" t="n">
+        <v>5</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>10035</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Imã 15</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>3</v>
+      </c>
+      <c r="E188" t="n">
+        <v>15</v>
+      </c>
+      <c r="F188" t="n">
+        <v>45</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>3</v>
+      </c>
+      <c r="E189" t="n">
+        <v>20</v>
+      </c>
+      <c r="F189" t="n">
+        <v>60</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>10013</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Oxe XG</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>1</v>
+      </c>
+      <c r="E190" t="n">
+        <v>65</v>
+      </c>
+      <c r="F190" t="n">
+        <v>65</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+      <c r="E191" t="n">
+        <v>20</v>
+      </c>
+      <c r="F191" t="n">
+        <v>20</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>21</v>
+      </c>
+      <c r="E192" t="n">
+        <v>55</v>
+      </c>
+      <c r="F192" t="n">
+        <v>1155</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>10015</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Regional infantil</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>2</v>
+      </c>
+      <c r="E193" t="n">
+        <v>45</v>
+      </c>
+      <c r="F193" t="n">
+        <v>90</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>item-sales-summary-2026-04-27-2026-04-27</t>
         </is>
       </c>
     </row>
@@ -11523,7 +12027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -12753,6 +13257,36 @@
         <v>3860</v>
       </c>
       <c r="F41" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Vendas 2026-04-27 → 2026-04-27</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>2050</v>
+      </c>
+      <c r="F42" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
data sync: 2026-06-22 11:51
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Cashflow" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="CategoryOverrides" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Meta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SupplierCatalog" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="PurchaseOrders" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2436,31 +2438,31 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>10041</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>Ima promoção 20 reais</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>Sem categoria</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="2" t="n">
         <v>7.5</v>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G75" s="2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2552,6 +2554,11 @@
       <c r="F2" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="n">
         <v>7</v>
       </c>
@@ -2586,6 +2593,11 @@
       <c r="F3" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="n">
         <v>7</v>
       </c>
@@ -2620,6 +2632,11 @@
       <c r="F4" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n">
         <v>7</v>
       </c>
@@ -2654,6 +2671,11 @@
       <c r="F5" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="n">
         <v>7</v>
       </c>
@@ -2688,6 +2710,11 @@
       <c r="F6" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="n">
         <v>7</v>
       </c>
@@ -2722,6 +2749,11 @@
       <c r="F7" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="n">
         <v>7</v>
       </c>
@@ -2756,6 +2788,11 @@
       <c r="F8" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="n">
         <v>7</v>
       </c>
@@ -2790,6 +2827,11 @@
       <c r="F9" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="n">
         <v>7</v>
       </c>
@@ -2824,6 +2866,11 @@
       <c r="F10" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="n">
         <v>7</v>
       </c>
@@ -2858,6 +2905,11 @@
       <c r="F11" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="n">
         <v>7</v>
       </c>
@@ -2892,6 +2944,11 @@
       <c r="F12" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="n">
         <v>7</v>
       </c>
@@ -2926,6 +2983,11 @@
       <c r="F13" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="n">
         <v>7</v>
       </c>
@@ -2960,6 +3022,11 @@
       <c r="F14" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="n">
         <v>7</v>
       </c>
@@ -2994,6 +3061,11 @@
       <c r="F15" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="n">
         <v>7</v>
       </c>
@@ -3028,6 +3100,11 @@
       <c r="F16" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="n">
         <v>7</v>
       </c>
@@ -3062,6 +3139,11 @@
       <c r="F17" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="n">
         <v>7</v>
       </c>
@@ -3096,6 +3178,11 @@
       <c r="F18" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="n">
         <v>7</v>
       </c>
@@ -3130,6 +3217,11 @@
       <c r="F19" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="n">
         <v>7</v>
       </c>
@@ -3164,6 +3256,11 @@
       <c r="F20" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="n">
         <v>7</v>
       </c>
@@ -3198,6 +3295,11 @@
       <c r="F21" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="n">
         <v>7</v>
       </c>
@@ -3232,6 +3334,11 @@
       <c r="F22" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="n">
         <v>7</v>
       </c>
@@ -3266,6 +3373,11 @@
       <c r="F23" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="n">
         <v>7</v>
       </c>
@@ -3300,6 +3412,11 @@
       <c r="F24" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="n">
         <v>7</v>
       </c>
@@ -3334,6 +3451,11 @@
       <c r="F25" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="n">
         <v>7</v>
       </c>
@@ -3368,6 +3490,11 @@
       <c r="F26" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="n">
         <v>7</v>
       </c>
@@ -3402,6 +3529,11 @@
       <c r="F27" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n">
         <v>7</v>
       </c>
@@ -3436,6 +3568,11 @@
       <c r="F28" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="n">
         <v>7</v>
       </c>
@@ -3470,6 +3607,11 @@
       <c r="F29" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="n">
         <v>7</v>
       </c>
@@ -3504,6 +3646,11 @@
       <c r="F30" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H30" s="2" t="n">
         <v>7</v>
       </c>
@@ -3538,6 +3685,11 @@
       <c r="F31" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="n">
         <v>7</v>
       </c>
@@ -3572,6 +3724,11 @@
       <c r="F32" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="n">
         <v>7</v>
       </c>
@@ -3606,6 +3763,11 @@
       <c r="F33" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H33" s="2" t="n">
         <v>7</v>
       </c>
@@ -3640,6 +3802,11 @@
       <c r="F34" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H34" s="2" t="n">
         <v>7</v>
       </c>
@@ -3674,6 +3841,11 @@
       <c r="F35" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H35" s="2" t="n">
         <v>7</v>
       </c>
@@ -3708,6 +3880,11 @@
       <c r="F36" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H36" s="2" t="n">
         <v>7</v>
       </c>
@@ -3742,6 +3919,11 @@
       <c r="F37" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H37" s="2" t="n">
         <v>7</v>
       </c>
@@ -3776,6 +3958,11 @@
       <c r="F38" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="n">
         <v>7</v>
       </c>
@@ -3810,6 +3997,11 @@
       <c r="F39" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H39" s="2" t="n">
         <v>7</v>
       </c>
@@ -3843,6 +4035,11 @@
       </c>
       <c r="F40" s="2" t="n">
         <v>15</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
       </c>
       <c r="H40" s="2" t="n">
         <v>7</v>
@@ -3876,7 +4073,11 @@
       <c r="F41" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H41" s="2" t="n">
         <v>7</v>
       </c>
@@ -3909,7 +4110,11 @@
       <c r="F42" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H42" s="2" t="n">
         <v>7</v>
       </c>
@@ -3942,7 +4147,11 @@
       <c r="F43" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H43" s="2" t="n">
         <v>7</v>
       </c>
@@ -3975,7 +4184,11 @@
       <c r="F44" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H44" s="2" t="n">
         <v>7</v>
       </c>
@@ -4008,7 +4221,11 @@
       <c r="F45" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H45" s="2" t="n">
         <v>7</v>
       </c>
@@ -4041,7 +4258,11 @@
       <c r="F46" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H46" s="2" t="n">
         <v>7</v>
       </c>
@@ -4074,7 +4295,11 @@
       <c r="F47" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H47" s="2" t="n">
         <v>7</v>
       </c>
@@ -4107,7 +4332,11 @@
       <c r="F48" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H48" s="2" t="n">
         <v>7</v>
       </c>
@@ -4140,7 +4369,11 @@
       <c r="F49" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H49" s="2" t="n">
         <v>7</v>
       </c>
@@ -4173,7 +4406,11 @@
       <c r="F50" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H50" s="2" t="n">
         <v>7</v>
       </c>
@@ -4206,7 +4443,11 @@
       <c r="F51" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H51" s="2" t="n">
         <v>7</v>
       </c>
@@ -4239,7 +4480,11 @@
       <c r="F52" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H52" s="2" t="n">
         <v>7</v>
       </c>
@@ -4272,7 +4517,11 @@
       <c r="F53" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H53" s="2" t="n">
         <v>7</v>
       </c>
@@ -4305,7 +4554,11 @@
       <c r="F54" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H54" s="2" t="n">
         <v>7</v>
       </c>
@@ -4338,7 +4591,11 @@
       <c r="F55" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H55" s="2" t="n">
         <v>7</v>
       </c>
@@ -4371,7 +4628,11 @@
       <c r="F56" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H56" s="2" t="n">
         <v>7</v>
       </c>
@@ -4404,7 +4665,11 @@
       <c r="F57" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H57" s="2" t="n">
         <v>7</v>
       </c>
@@ -4437,7 +4702,11 @@
       <c r="F58" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H58" s="2" t="n">
         <v>7</v>
       </c>
@@ -4470,7 +4739,11 @@
       <c r="F59" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H59" s="2" t="n">
         <v>7</v>
       </c>
@@ -4503,7 +4776,11 @@
       <c r="F60" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H60" s="2" t="n">
         <v>7</v>
       </c>
@@ -4536,7 +4813,11 @@
       <c r="F61" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H61" s="2" t="n">
         <v>7</v>
       </c>
@@ -4569,7 +4850,11 @@
       <c r="F62" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H62" s="2" t="n">
         <v>7</v>
       </c>
@@ -4602,7 +4887,11 @@
       <c r="F63" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H63" s="2" t="n">
         <v>7</v>
       </c>
@@ -4635,7 +4924,11 @@
       <c r="F64" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H64" s="2" t="n">
         <v>7</v>
       </c>
@@ -4668,7 +4961,11 @@
       <c r="F65" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H65" s="2" t="n">
         <v>7</v>
       </c>
@@ -4701,7 +4998,11 @@
       <c r="F66" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H66" s="2" t="n">
         <v>7</v>
       </c>
@@ -4734,7 +5035,11 @@
       <c r="F67" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H67" s="2" t="n">
         <v>7</v>
       </c>
@@ -4767,7 +5072,11 @@
       <c r="F68" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H68" s="2" t="n">
         <v>7</v>
       </c>
@@ -4800,7 +5109,11 @@
       <c r="F69" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
       <c r="H69" s="2" t="n">
         <v>7</v>
       </c>
@@ -4833,7 +5146,11 @@
       <c r="F70" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
       <c r="H70" s="2" t="n">
         <v>7</v>
       </c>
@@ -4866,7 +5183,11 @@
       <c r="F71" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
       <c r="H71" s="2" t="n">
         <v>7</v>
       </c>
@@ -4899,7 +5220,11 @@
       <c r="F72" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
       <c r="H72" s="2" t="n">
         <v>7</v>
       </c>
@@ -4934,6 +5259,11 @@
       <c r="F73" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
       <c r="H73" s="2" t="n">
         <v>7</v>
       </c>
@@ -4968,40 +5298,49 @@
       <c r="F74" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
       <c r="H74" s="2" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>10041</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>Ima promoção 20 reais</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>Sem categoria</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H75" t="n">
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>Added during Jun 2026 Loyverse backfill</t>
         </is>
@@ -20878,4 +21217,2045 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>supplier_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>supplier_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>lead_time_days</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>moq</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>case_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>21</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10004</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10006</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>21</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10008</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10009</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>10010</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>21</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>10011</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10012</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>21</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10013</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>21</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>21</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10015</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>21</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10016</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>21</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10017</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10018</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ALGODOEIRO ECO FASHION</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>21</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10020</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>45</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10021</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10022</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>45</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>45</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>45</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>45</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>10027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>45</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>14</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>10029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>14</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>14</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>14</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>10032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>14</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>10033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>14</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>14</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>10035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>14</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>14</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>10037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>14</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>14</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>45</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>00400</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>45</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6</v>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>00401</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>45</v>
+      </c>
+      <c r="E42" t="n">
+        <v>6</v>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>00402</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>45</v>
+      </c>
+      <c r="E43" t="n">
+        <v>6</v>
+      </c>
+      <c r="F43" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>00403</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>45</v>
+      </c>
+      <c r="E44" t="n">
+        <v>6</v>
+      </c>
+      <c r="F44" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>00404</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>45</v>
+      </c>
+      <c r="E45" t="n">
+        <v>6</v>
+      </c>
+      <c r="F45" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>00405</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>45</v>
+      </c>
+      <c r="E46" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>00406</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>45</v>
+      </c>
+      <c r="E47" t="n">
+        <v>6</v>
+      </c>
+      <c r="F47" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>00407</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>45</v>
+      </c>
+      <c r="E48" t="n">
+        <v>6</v>
+      </c>
+      <c r="F48" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>00408</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>45</v>
+      </c>
+      <c r="E49" t="n">
+        <v>6</v>
+      </c>
+      <c r="F49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>00409</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>45</v>
+      </c>
+      <c r="E50" t="n">
+        <v>6</v>
+      </c>
+      <c r="F50" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>00410</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>45</v>
+      </c>
+      <c r="E51" t="n">
+        <v>6</v>
+      </c>
+      <c r="F51" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>00411</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>45</v>
+      </c>
+      <c r="E52" t="n">
+        <v>6</v>
+      </c>
+      <c r="F52" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>00412</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>45</v>
+      </c>
+      <c r="E53" t="n">
+        <v>6</v>
+      </c>
+      <c r="F53" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>00413</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>45</v>
+      </c>
+      <c r="E54" t="n">
+        <v>6</v>
+      </c>
+      <c r="F54" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>00414</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>45</v>
+      </c>
+      <c r="E55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F55" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>00415</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>45</v>
+      </c>
+      <c r="E56" t="n">
+        <v>6</v>
+      </c>
+      <c r="F56" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>00416</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>45</v>
+      </c>
+      <c r="E57" t="n">
+        <v>6</v>
+      </c>
+      <c r="F57" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>00417</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>45</v>
+      </c>
+      <c r="E58" t="n">
+        <v>6</v>
+      </c>
+      <c r="F58" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>00418</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>45</v>
+      </c>
+      <c r="E59" t="n">
+        <v>6</v>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>00419</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>45</v>
+      </c>
+      <c r="E60" t="n">
+        <v>6</v>
+      </c>
+      <c r="F60" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>00420</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>45</v>
+      </c>
+      <c r="E61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F61" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>00421</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>45</v>
+      </c>
+      <c r="E62" t="n">
+        <v>6</v>
+      </c>
+      <c r="F62" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>00422</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>45</v>
+      </c>
+      <c r="E63" t="n">
+        <v>6</v>
+      </c>
+      <c r="F63" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>00423</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>45</v>
+      </c>
+      <c r="E64" t="n">
+        <v>6</v>
+      </c>
+      <c r="F64" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>00424</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>45</v>
+      </c>
+      <c r="E65" t="n">
+        <v>6</v>
+      </c>
+      <c r="F65" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>00425</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>45</v>
+      </c>
+      <c r="E66" t="n">
+        <v>6</v>
+      </c>
+      <c r="F66" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>00426</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>45</v>
+      </c>
+      <c r="E67" t="n">
+        <v>6</v>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>00427</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>45</v>
+      </c>
+      <c r="E68" t="n">
+        <v>6</v>
+      </c>
+      <c r="F68" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>00428</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>30</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>00429</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>30</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>00430</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>30</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>00431</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>GIRISH INDIANA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>30</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>10040</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>14</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>10024</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ALAN BOLSAS</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>45</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>10041</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDOR (GENÉRICO)</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>14</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>po_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>supplier_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>supplier_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>unit_cost</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>line_total</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
data: add sales Jun 20-21 2026 via Loyverse automation
Jun 20: R$ 4,075 (21 SKUs)
Jun 21: R$ 3,264 (20 SKUs)
Coverage now 2026-04-29 → 2026-06-21

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -5355,7 +5355,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H415"/>
+  <dimension ref="A1:H456"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -20301,6 +20301,1482 @@
       <c r="H415" t="inlineStr">
         <is>
           <t>loyverse_reconcile_item_sales_summary_2026-03-01_2026-06-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>10022</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Bolsinha 15</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E416" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="F416" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Caneca louça</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="E417" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="F417" t="n">
+        <v>385.0</v>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="E418" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F418" t="n">
+        <v>200.0</v>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>10029</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 30</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E419" t="n">
+        <v>30.0</v>
+      </c>
+      <c r="F419" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E420" t="n">
+        <v>55.0</v>
+      </c>
+      <c r="F420" t="n">
+        <v>55.0</v>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>10006</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Canga viscose</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E421" t="n">
+        <v>65.0</v>
+      </c>
+      <c r="F421" t="n">
+        <v>65.0</v>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Carteira alça</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="E422" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="F422" t="n">
+        <v>45.0</v>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>54.0</v>
+      </c>
+      <c r="E423" t="n">
+        <v>9.814814814814815</v>
+      </c>
+      <c r="F423" t="n">
+        <v>530.0</v>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>10007</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Color 60</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E424" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="F424" t="n">
+        <v>120.0</v>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Ecobag</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="E425" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="F425" t="n">
+        <v>150.0</v>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>10037</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Embalagem presente 10</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E426" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="F426" t="n">
+        <v>14.0</v>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Embalagem presente 5</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E427" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="F427" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>10041</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Ima promoção 20 reais</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E428" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F428" t="n">
+        <v>40.0</v>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>10009</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Macaquinho</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E429" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="F429" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="E430" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F430" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="E431" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F431" t="n">
+        <v>340.0</v>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Placa kit 100</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E432" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="F432" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="E433" t="n">
+        <v>55.0</v>
+      </c>
+      <c r="F433" t="n">
+        <v>825.0</v>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>10015</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Regional infantil</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E434" t="n">
+        <v>45.0</v>
+      </c>
+      <c r="F434" t="n">
+        <v>45.0</v>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>10016</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Saída praia</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E435" t="n">
+        <v>65.0</v>
+      </c>
+      <c r="F435" t="n">
+        <v>65.0</v>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-21_2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="E436" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="F436" t="n">
+        <v>140.0</v>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>10004</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Body conjunto</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E437" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="F437" t="n">
+        <v>120.0</v>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>10039</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Bolsa kit 125</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="E438" t="n">
+        <v>125.0</v>
+      </c>
+      <c r="F438" t="n">
+        <v>875.0</v>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>10032</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Boneca</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E439" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="F439" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>10040</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Boneca oxe</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E440" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="F440" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>10031</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Boné</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E441" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="F441" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>10030</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Caneca louça</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="E442" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="F442" t="n">
+        <v>105.0</v>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>10028</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Caneca Ágata 20</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E443" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F443" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>10005</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Canga elastano</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="E444" t="n">
+        <v>55.0</v>
+      </c>
+      <c r="F444" t="n">
+        <v>220.0</v>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>10023</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Carteira alça</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="E445" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="F445" t="n">
+        <v>75.0</v>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>10034</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Chaveiro ímã 10</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>34.0</v>
+      </c>
+      <c r="E446" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="F446" t="n">
+        <v>340.0</v>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>10025</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Ecobag</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E447" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="F447" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>10041</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Ima promoção 20 reais</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="E448" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F448" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>10009</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Macaquinho</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E449" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="F449" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>10026</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Necessaire</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>9.0</v>
+      </c>
+      <c r="E450" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F450" t="n">
+        <v>180.0</v>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>10010</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Oxe adulto</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E451" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="F451" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>10012</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Oxe conjunto</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E452" t="n">
+        <v>80.0</v>
+      </c>
+      <c r="F452" t="n">
+        <v>80.0</v>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>10019</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="E453" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="F453" t="n">
+        <v>140.0</v>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>10038</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Placa kit 100</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E454" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="F454" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>10014</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Regional adulto</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="E455" t="n">
+        <v>55.0</v>
+      </c>
+      <c r="F455" t="n">
+        <v>1210.0</v>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>10016</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Saída praia</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E456" t="n">
+        <v>65.0</v>
+      </c>
+      <c r="F456" t="n">
+        <v>130.0</v>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>item_sales_summary_2026-06-20_2026-06-20</t>
         </is>
       </c>
     </row>
@@ -20310,7 +21786,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -21120,6 +22596,126 @@
         <v>123835.84999999999</v>
       </c>
       <c r="F27" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Vendas 2026-06-21 -&gt; 2026-06-21</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>3264.0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CMV</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CMV 2026-06-21 -&gt; 2026-06-21</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1390.7</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Vendas</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Vendas 2026-06-20 -&gt; 2026-06-20</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>4075.0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CMV</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CMV 2026-06-20 -&gt; 2026-06-20</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1755.05</v>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>Misto</t>
         </is>

</xml_diff>

<commit_message>
data sync: 2026-07-29 07:17
</commit_message>
<xml_diff>
--- a/data/excel/FuloFilo_Master.xlsx
+++ b/data/excel/FuloFilo_Master.xlsx
@@ -37079,7 +37079,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Vendas 2026-07-11 -&gt; 2026-07-11</t>
+          <t>Loyverse anchor 2026-07-11 -&gt; 2026-07-11</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -37109,7 +37109,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>CMV 2026-07-11 -&gt; 2026-07-11</t>
+          <t>Loyverse anchor CMV 2026-07-11 -&gt; 2026-07-11</t>
         </is>
       </c>
       <c r="E67" t="n">

</xml_diff>